<commit_message>
Deploy data to app repo
</commit_message>
<xml_diff>
--- a/data/xlsx/Baernreither_Index_2023.xlsx
+++ b/data/xlsx/Baernreither_Index_2023.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christofaichner/Documents/GitHub/baernreither-data/data/xlsx/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/melaniedaubner/Documents/baernreither-data/data/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A68E3AA-8331-5340-999E-E77B2C20F82E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{683B84D5-2003-4147-8B93-168E38D41A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="320" yWindow="2100" windowWidth="25600" windowHeight="14760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="338">
   <si>
     <t>Hauptbegriff</t>
   </si>
@@ -975,16 +975,98 @@
   <si>
     <t>&lt;index&gt;&lt;term key="Weltausstellung"&gt; &lt;/term&gt;&lt;/index&gt;</t>
   </si>
+  <si>
+    <t>Vollzugsausschuss</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="Parteien"&gt;  &lt;/term&gt;&lt;index&gt;&lt;term key="Vollzugsausschuss"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>Zucker Kontingentierung</t>
+  </si>
+  <si>
+    <t>ZuckerKontingentierung</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="ZuckerKontingentierung"&gt;       &lt;/term&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>Zuckerfrage</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="Zuckerfrage"&gt;       &lt;/term&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>Vereinigtes Königreich</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolonialpolitik </t>
+  </si>
+  <si>
+    <t>VereinigtesKoenigreich</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="VereinigtesKoenigreich"&gt;  &lt;/term&gt;&lt;index&gt;&lt;term key="Kolonialpolitik"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>Zollpolitik</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="VereinigtesKoenigreich"&gt;  &lt;/term&gt;&lt;index&gt;&lt;term key="Zollpolitik"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>Internationale Brüsseler Zuckerkonvention</t>
+  </si>
+  <si>
+    <t>InternationaleBruesselerZuckerkonvention</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="InternationaleBruesselerZuckerkonvention"&gt;    &lt;/term&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>Brüsseler Konferenz</t>
+  </si>
+  <si>
+    <t>BruesselerKonferenz</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="InternationaleBruesselerZuckerkonvention"&gt;    &lt;/term&gt;&lt;index&gt;&lt;term key="BruesselerKonferenz"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>Kanada</t>
+  </si>
+  <si>
+    <t>Nationalitätenfrage</t>
+  </si>
+  <si>
+    <t>Nationalitaetenfrage</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="Kanada"&gt;   &lt;/term&gt;&lt;index&gt;&lt;term key="Nationalitaetenfrage"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="Kanada"&gt;   &lt;/term&gt;&lt;index&gt;&lt;term key="Zolltarif"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
+  </si>
+  <si>
+    <t>&lt;index&gt;&lt;term key="Kanada"&gt;   &lt;/term&gt;&lt;index&gt;&lt;term key="Sprachenfrage"/&gt;&lt;/index&gt;&lt;/index&gt;</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1017,7 +1099,7 @@
       <name val="&quot;Helvetica Neue&quot;"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1060,6 +1142,24 @@
         <bgColor theme="7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDB9CFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDB9CFF"/>
+        <bgColor rgb="FFC27BA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDB9CFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1082,62 +1182,81 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1353,7 +1472,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC1053"/>
+  <dimension ref="A1:AC1061"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="34.5" style="4" customWidth="1"/>
@@ -2404,16 +2523,16 @@
       <c r="AC27" s="3"/>
     </row>
     <row r="28" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A28" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="16" t="s">
-        <v>275</v>
-      </c>
-      <c r="D28" s="17"/>
-      <c r="E28" s="13" t="s">
-        <v>276</v>
+      <c r="A28" s="33" t="s">
+        <v>326</v>
+      </c>
+      <c r="B28" s="34"/>
+      <c r="C28" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="D28" s="34"/>
+      <c r="E28" s="28" t="s">
+        <v>328</v>
       </c>
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
@@ -2441,20 +2560,20 @@
       <c r="AC28" s="3"/>
     </row>
     <row r="29" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A29" s="18" t="s">
-        <v>59</v>
-      </c>
-      <c r="B29" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="C29" s="18" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>62</v>
+      <c r="A29" s="33" t="s">
+        <v>326</v>
+      </c>
+      <c r="B29" s="34" t="s">
+        <v>329</v>
+      </c>
+      <c r="C29" s="33" t="s">
+        <v>327</v>
+      </c>
+      <c r="D29" s="34" t="s">
+        <v>330</v>
+      </c>
+      <c r="E29" s="28" t="s">
+        <v>331</v>
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
@@ -2482,20 +2601,16 @@
       <c r="AC29" s="3"/>
     </row>
     <row r="30" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A30" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>277</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="D30" s="19" t="s">
-        <v>277</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>278</v>
+      <c r="A30" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="D30" s="17"/>
+      <c r="E30" s="13" t="s">
+        <v>276</v>
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
@@ -2523,20 +2638,20 @@
       <c r="AC30" s="3"/>
     </row>
     <row r="31" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A31" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>279</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>279</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>280</v>
+      <c r="A31" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="B31" s="28" t="s">
+        <v>333</v>
+      </c>
+      <c r="C31" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="D31" s="28" t="s">
+        <v>334</v>
+      </c>
+      <c r="E31" s="28" t="s">
+        <v>335</v>
       </c>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
@@ -2564,20 +2679,20 @@
       <c r="AC31" s="3"/>
     </row>
     <row r="32" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A32" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>269</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>66</v>
+      <c r="A32" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="B32" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="C32" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="D32" s="28" t="s">
+        <v>46</v>
+      </c>
+      <c r="E32" s="28" t="s">
+        <v>336</v>
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
@@ -2605,20 +2720,20 @@
       <c r="AC32" s="3"/>
     </row>
     <row r="33" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A33" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>69</v>
+      <c r="A33" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="B33" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C33" s="35" t="s">
+        <v>332</v>
+      </c>
+      <c r="D33" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="E33" s="28" t="s">
+        <v>337</v>
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
@@ -2646,16 +2761,20 @@
       <c r="AC33" s="3"/>
     </row>
     <row r="34" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A34" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B34" s="3"/>
-      <c r="C34" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D34" s="3"/>
+      <c r="A34" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>60</v>
+      </c>
       <c r="E34" s="3" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
@@ -2683,16 +2802,20 @@
       <c r="AC34" s="3"/>
     </row>
     <row r="35" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A35" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D35" s="3"/>
+      <c r="A35" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>277</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>277</v>
+      </c>
       <c r="E35" s="3" t="s">
-        <v>73</v>
+        <v>278</v>
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
@@ -2720,16 +2843,20 @@
       <c r="AC35" s="3"/>
     </row>
     <row r="36" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A36" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B36" s="3"/>
-      <c r="C36" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D36" s="3"/>
+      <c r="A36" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>279</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>279</v>
+      </c>
       <c r="E36" s="3" t="s">
-        <v>76</v>
+        <v>280</v>
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
@@ -2757,20 +2884,20 @@
       <c r="AC36" s="3"/>
     </row>
     <row r="37" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A37" s="1" t="s">
-        <v>74</v>
+      <c r="A37" s="20" t="s">
+        <v>63</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>75</v>
+        <v>64</v>
+      </c>
+      <c r="C37" s="20" t="s">
+        <v>269</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
@@ -2798,20 +2925,20 @@
       <c r="AC37" s="3"/>
     </row>
     <row r="38" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A38" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D38" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>81</v>
+      <c r="A38" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>69</v>
       </c>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
@@ -2839,20 +2966,16 @@
       <c r="AC38" s="3"/>
     </row>
     <row r="39" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A39" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="B39" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D39" s="10" t="s">
-        <v>83</v>
-      </c>
+      <c r="A39" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D39" s="3"/>
       <c r="E39" s="3" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
@@ -2880,20 +3003,16 @@
       <c r="AC39" s="3"/>
     </row>
     <row r="40" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A40" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>281</v>
-      </c>
-      <c r="C40" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="D40" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="E40" s="13" t="s">
-        <v>282</v>
+      <c r="A40" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B40" s="3"/>
+      <c r="C40" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3" t="s">
+        <v>73</v>
       </c>
       <c r="F40" s="3"/>
       <c r="G40" s="3"/>
@@ -2922,19 +3041,15 @@
     </row>
     <row r="41" spans="1:29" ht="15.75" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>57</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="B41" s="3"/>
       <c r="C41" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D41" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E41" s="21" t="s">
-        <v>87</v>
+        <v>75</v>
+      </c>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3" t="s">
+        <v>76</v>
       </c>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
@@ -2962,20 +3077,20 @@
       <c r="AC41" s="3"/>
     </row>
     <row r="42" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A42" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="B42" s="10" t="s">
-        <v>88</v>
+      <c r="A42" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>77</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="D42" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="E42" s="21" t="s">
-        <v>89</v>
+        <v>75</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>78</v>
       </c>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
@@ -3003,20 +3118,20 @@
       <c r="AC42" s="3"/>
     </row>
     <row r="43" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A43" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="E43" s="22" t="s">
-        <v>92</v>
+      <c r="A43" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>81</v>
       </c>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
@@ -3044,20 +3159,20 @@
       <c r="AC43" s="3"/>
     </row>
     <row r="44" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A44" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="B44" s="13" t="s">
-        <v>283</v>
-      </c>
-      <c r="C44" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="D44" s="13" t="s">
-        <v>284</v>
-      </c>
-      <c r="E44" s="22" t="s">
-        <v>285</v>
+      <c r="A44" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>84</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="3"/>
@@ -3085,20 +3200,20 @@
       <c r="AC44" s="3"/>
     </row>
     <row r="45" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A45" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="B45" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D45" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="E45" s="22" t="s">
-        <v>94</v>
+      <c r="A45" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>281</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="E45" s="13" t="s">
+        <v>282</v>
       </c>
       <c r="F45" s="3"/>
       <c r="G45" s="3"/>
@@ -3126,20 +3241,20 @@
       <c r="AC45" s="3"/>
     </row>
     <row r="46" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A46" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="B46" s="10" t="s">
-        <v>95</v>
+      <c r="A46" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D46" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="E46" s="22" t="s">
-        <v>96</v>
+        <v>86</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="E46" s="21" t="s">
+        <v>87</v>
       </c>
       <c r="F46" s="3"/>
       <c r="G46" s="3"/>
@@ -3167,20 +3282,20 @@
       <c r="AC46" s="3"/>
     </row>
     <row r="47" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A47" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>33</v>
+      <c r="A47" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B47" s="10" t="s">
+        <v>88</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D47" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="E47" s="22" t="s">
-        <v>97</v>
+        <v>86</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="E47" s="21" t="s">
+        <v>89</v>
       </c>
       <c r="F47" s="3"/>
       <c r="G47" s="3"/>
@@ -3208,20 +3323,20 @@
       <c r="AC47" s="3"/>
     </row>
     <row r="48" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B48" s="13" t="s">
-        <v>286</v>
-      </c>
-      <c r="C48" s="12" t="s">
+      <c r="B48" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D48" s="13" t="s">
-        <v>287</v>
-      </c>
-      <c r="E48" s="13" t="s">
-        <v>288</v>
+      <c r="D48" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E48" s="22" t="s">
+        <v>92</v>
       </c>
       <c r="F48" s="3"/>
       <c r="G48" s="3"/>
@@ -3249,20 +3364,20 @@
       <c r="AC48" s="3"/>
     </row>
     <row r="49" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A49" s="1" t="s">
+      <c r="A49" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B49" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C49" s="1" t="s">
+      <c r="B49" s="13" t="s">
+        <v>283</v>
+      </c>
+      <c r="C49" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>99</v>
+      <c r="D49" s="13" t="s">
+        <v>284</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>100</v>
+        <v>285</v>
       </c>
       <c r="F49" s="3"/>
       <c r="G49" s="3"/>
@@ -3294,16 +3409,16 @@
         <v>90</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>101</v>
+        <v>93</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D50" s="10" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>103</v>
+        <v>94</v>
       </c>
       <c r="F50" s="3"/>
       <c r="G50" s="3"/>
@@ -3335,16 +3450,16 @@
         <v>90</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>57</v>
+        <v>95</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>57</v>
+        <v>95</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>104</v>
+        <v>96</v>
       </c>
       <c r="F51" s="3"/>
       <c r="G51" s="3"/>
@@ -3376,16 +3491,16 @@
         <v>90</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>105</v>
+        <v>33</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="E52" s="3" t="s">
-        <v>106</v>
+        <v>33</v>
+      </c>
+      <c r="E52" s="22" t="s">
+        <v>97</v>
       </c>
       <c r="F52" s="3"/>
       <c r="G52" s="3"/>
@@ -3413,20 +3528,20 @@
       <c r="AC52" s="3"/>
     </row>
     <row r="53" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A53" s="1" t="s">
+      <c r="A53" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="B53" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C53" s="1" t="s">
+      <c r="B53" s="13" t="s">
+        <v>286</v>
+      </c>
+      <c r="C53" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D53" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>108</v>
+      <c r="D53" s="13" t="s">
+        <v>287</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>288</v>
       </c>
       <c r="F53" s="3"/>
       <c r="G53" s="3"/>
@@ -3458,16 +3573,16 @@
         <v>90</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>109</v>
+        <v>98</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>110</v>
+        <v>99</v>
+      </c>
+      <c r="E54" s="22" t="s">
+        <v>100</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
@@ -3495,20 +3610,20 @@
       <c r="AC54" s="3"/>
     </row>
     <row r="55" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A55" s="1" t="s">
+      <c r="A55" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B55" s="3" t="s">
-        <v>111</v>
+      <c r="B55" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D55" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E55" s="3" t="s">
-        <v>113</v>
+      <c r="D55" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="E55" s="22" t="s">
+        <v>103</v>
       </c>
       <c r="F55" s="3"/>
       <c r="G55" s="3"/>
@@ -3536,20 +3651,20 @@
       <c r="AC55" s="3"/>
     </row>
     <row r="56" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A56" s="1" t="s">
+      <c r="A56" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B56" s="3" t="s">
-        <v>114</v>
+      <c r="B56" s="10" t="s">
+        <v>57</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D56" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>116</v>
+      <c r="D56" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="E56" s="22" t="s">
+        <v>104</v>
       </c>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -3581,16 +3696,16 @@
         <v>90</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>119</v>
+        <v>106</v>
       </c>
       <c r="F57" s="3"/>
       <c r="G57" s="3"/>
@@ -3622,16 +3737,16 @@
         <v>90</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="F58" s="3"/>
       <c r="G58" s="3"/>
@@ -3659,20 +3774,20 @@
       <c r="AC58" s="3"/>
     </row>
     <row r="59" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B59" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="C59" s="12" t="s">
+      <c r="B59" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C59" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D59" s="13" t="s">
-        <v>289</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>290</v>
+      <c r="D59" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>110</v>
       </c>
       <c r="F59" s="3"/>
       <c r="G59" s="3"/>
@@ -3704,16 +3819,16 @@
         <v>90</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>46</v>
+        <v>111</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>46</v>
+        <v>112</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
       <c r="F60" s="3"/>
       <c r="G60" s="3"/>
@@ -3745,16 +3860,16 @@
         <v>90</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>91</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="F61" s="3"/>
       <c r="G61" s="3"/>
@@ -3782,16 +3897,20 @@
       <c r="AC61" s="3"/>
     </row>
     <row r="62" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A62" s="12" t="s">
-        <v>291</v>
-      </c>
-      <c r="B62" s="13"/>
-      <c r="C62" s="12" t="s">
-        <v>291</v>
-      </c>
-      <c r="D62" s="13"/>
-      <c r="E62" s="13" t="s">
-        <v>292</v>
+      <c r="A62" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E62" s="3" t="s">
+        <v>119</v>
       </c>
       <c r="F62" s="3"/>
       <c r="G62" s="3"/>
@@ -3820,15 +3939,19 @@
     </row>
     <row r="63" spans="1:29" ht="15.75" customHeight="1">
       <c r="A63" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="B63" s="3"/>
+        <v>90</v>
+      </c>
+      <c r="B63" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="C63" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D63" s="3"/>
+        <v>91</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="E63" s="3" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="F63" s="3"/>
       <c r="G63" s="3"/>
@@ -3857,15 +3980,19 @@
     </row>
     <row r="64" spans="1:29" ht="15.75" customHeight="1">
       <c r="A64" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="B64" s="13"/>
+        <v>90</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>289</v>
+      </c>
       <c r="C64" s="12" t="s">
-        <v>293</v>
-      </c>
-      <c r="D64" s="13"/>
-      <c r="E64" s="13" t="s">
-        <v>294</v>
+        <v>91</v>
+      </c>
+      <c r="D64" s="13" t="s">
+        <v>289</v>
+      </c>
+      <c r="E64" s="22" t="s">
+        <v>290</v>
       </c>
       <c r="F64" s="3"/>
       <c r="G64" s="3"/>
@@ -3894,15 +4021,19 @@
     </row>
     <row r="65" spans="1:29" ht="15.75" customHeight="1">
       <c r="A65" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B65" s="3"/>
+        <v>90</v>
+      </c>
+      <c r="B65" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="C65" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D65" s="3"/>
+        <v>91</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>46</v>
+      </c>
       <c r="E65" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="F65" s="3"/>
       <c r="G65" s="3"/>
@@ -3931,19 +4062,19 @@
     </row>
     <row r="66" spans="1:29" ht="15.75" customHeight="1">
       <c r="A66" s="1" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="F66" s="3"/>
       <c r="G66" s="3"/>
@@ -3971,20 +4102,16 @@
       <c r="AC66" s="3"/>
     </row>
     <row r="67" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A67" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B67" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>134</v>
+      <c r="A67" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="B67" s="13"/>
+      <c r="C67" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="D67" s="13"/>
+      <c r="E67" s="13" t="s">
+        <v>292</v>
       </c>
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
@@ -4013,19 +4140,15 @@
     </row>
     <row r="68" spans="1:29" ht="15.75" customHeight="1">
       <c r="A68" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="B68" s="3" t="s">
-        <v>135</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="B68" s="3"/>
       <c r="C68" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>136</v>
-      </c>
+        <v>125</v>
+      </c>
+      <c r="D68" s="3"/>
       <c r="E68" s="3" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F68" s="3"/>
       <c r="G68" s="3"/>
@@ -4053,20 +4176,16 @@
       <c r="AC68" s="3"/>
     </row>
     <row r="69" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A69" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="B69" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="C69" s="9" t="s">
-        <v>127</v>
-      </c>
-      <c r="D69" s="10" t="s">
-        <v>139</v>
-      </c>
-      <c r="E69" s="10" t="s">
-        <v>140</v>
+      <c r="A69" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="B69" s="13"/>
+      <c r="C69" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="D69" s="13"/>
+      <c r="E69" s="13" t="s">
+        <v>294</v>
       </c>
       <c r="F69" s="3"/>
       <c r="G69" s="3"/>
@@ -4094,20 +4213,16 @@
       <c r="AC69" s="3"/>
     </row>
     <row r="70" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A70" s="9" t="s">
+      <c r="A70" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B70" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="C70" s="9" t="s">
+      <c r="B70" s="3"/>
+      <c r="C70" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D70" s="10" t="s">
-        <v>141</v>
-      </c>
-      <c r="E70" s="10" t="s">
-        <v>142</v>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="F70" s="3"/>
       <c r="G70" s="3"/>
@@ -4135,20 +4250,20 @@
       <c r="AC70" s="3"/>
     </row>
     <row r="71" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A71" s="12" t="s">
+      <c r="A71" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B71" s="13" t="s">
-        <v>295</v>
-      </c>
-      <c r="C71" s="12" t="s">
+      <c r="B71" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C71" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D71" s="13" t="s">
-        <v>296</v>
-      </c>
-      <c r="E71" s="13" t="s">
-        <v>297</v>
+      <c r="D71" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E71" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="F71" s="3"/>
       <c r="G71" s="3"/>
@@ -4176,16 +4291,20 @@
       <c r="AC71" s="3"/>
     </row>
     <row r="72" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A72" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="B72" s="10"/>
-      <c r="C72" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="D72" s="10"/>
+      <c r="A72" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>133</v>
+      </c>
       <c r="E72" s="3" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="F72" s="3"/>
       <c r="G72" s="3"/>
@@ -4214,15 +4333,19 @@
     </row>
     <row r="73" spans="1:29" ht="15.75" customHeight="1">
       <c r="A73" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="B73" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="B73" s="3" t="s">
+        <v>135</v>
+      </c>
       <c r="C73" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D73" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>136</v>
+      </c>
       <c r="E73" s="3" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="F73" s="3"/>
       <c r="G73" s="3"/>
@@ -4250,20 +4373,20 @@
       <c r="AC73" s="3"/>
     </row>
     <row r="74" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A74" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="B74" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="C74" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="D74" s="13" t="s">
-        <v>298</v>
-      </c>
-      <c r="E74" s="13" t="s">
-        <v>299</v>
+      <c r="A74" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="B74" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="C74" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="D74" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="E74" s="28" t="s">
+        <v>314</v>
       </c>
       <c r="F74" s="3"/>
       <c r="G74" s="3"/>
@@ -4291,20 +4414,20 @@
       <c r="AC74" s="3"/>
     </row>
     <row r="75" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A75" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="B75" s="13" t="s">
-        <v>300</v>
-      </c>
-      <c r="C75" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="D75" s="13" t="s">
-        <v>300</v>
-      </c>
-      <c r="E75" s="13" t="s">
-        <v>301</v>
+      <c r="A75" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B75" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D75" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E75" s="10" t="s">
+        <v>140</v>
       </c>
       <c r="F75" s="3"/>
       <c r="G75" s="3"/>
@@ -4332,20 +4455,20 @@
       <c r="AC75" s="3"/>
     </row>
     <row r="76" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A76" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="B76" s="13" t="s">
-        <v>302</v>
-      </c>
-      <c r="C76" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="D76" s="13" t="s">
-        <v>303</v>
-      </c>
-      <c r="E76" s="13" t="s">
-        <v>304</v>
+      <c r="A76" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="B76" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="C76" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D76" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>142</v>
       </c>
       <c r="F76" s="3"/>
       <c r="G76" s="3"/>
@@ -4373,20 +4496,20 @@
       <c r="AC76" s="3"/>
     </row>
     <row r="77" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A77" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B77" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="E77" s="3" t="s">
-        <v>149</v>
+      <c r="A77" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B77" s="13" t="s">
+        <v>295</v>
+      </c>
+      <c r="C77" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D77" s="13" t="s">
+        <v>296</v>
+      </c>
+      <c r="E77" s="13" t="s">
+        <v>297</v>
       </c>
       <c r="F77" s="3"/>
       <c r="G77" s="3"/>
@@ -4415,19 +4538,15 @@
     </row>
     <row r="78" spans="1:29" ht="15.75" customHeight="1">
       <c r="A78" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="B78" s="10" t="s">
-        <v>150</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="B78" s="10"/>
       <c r="C78" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D78" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="E78" s="11" t="s">
-        <v>151</v>
+        <v>143</v>
+      </c>
+      <c r="D78" s="10"/>
+      <c r="E78" s="3" t="s">
+        <v>144</v>
       </c>
       <c r="F78" s="3"/>
       <c r="G78" s="3"/>
@@ -4455,20 +4574,16 @@
       <c r="AC78" s="3"/>
     </row>
     <row r="79" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A79" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="B79" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="C79" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D79" s="10" t="s">
-        <v>152</v>
-      </c>
+      <c r="A79" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B79" s="3"/>
+      <c r="C79" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D79" s="3"/>
       <c r="E79" s="3" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="F79" s="3"/>
       <c r="G79" s="3"/>
@@ -4496,20 +4611,20 @@
       <c r="AC79" s="3"/>
     </row>
     <row r="80" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A80" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B80" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="D80" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="E80" s="3" t="s">
-        <v>154</v>
+      <c r="A80" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B80" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="C80" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="E80" s="13" t="s">
+        <v>299</v>
       </c>
       <c r="F80" s="3"/>
       <c r="G80" s="3"/>
@@ -4537,20 +4652,20 @@
       <c r="AC80" s="3"/>
     </row>
     <row r="81" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A81" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="B81" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C81" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="D81" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="E81" s="3" t="s">
-        <v>157</v>
+      <c r="A81" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B81" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="C81" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="E81" s="13" t="s">
+        <v>301</v>
       </c>
       <c r="F81" s="3"/>
       <c r="G81" s="3"/>
@@ -4578,20 +4693,20 @@
       <c r="AC81" s="3"/>
     </row>
     <row r="82" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A82" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="B82" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="C82" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="D82" s="10" t="s">
-        <v>159</v>
-      </c>
-      <c r="E82" s="11" t="s">
-        <v>160</v>
+      <c r="A82" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B82" s="13" t="s">
+        <v>302</v>
+      </c>
+      <c r="C82" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="D82" s="13" t="s">
+        <v>303</v>
+      </c>
+      <c r="E82" s="13" t="s">
+        <v>304</v>
       </c>
       <c r="F82" s="3"/>
       <c r="G82" s="3"/>
@@ -4619,20 +4734,20 @@
       <c r="AC82" s="3"/>
     </row>
     <row r="83" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A83" s="9" t="s">
+      <c r="A83" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B83" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="C83" s="9" t="s">
+      <c r="B83" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C83" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D83" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="E83" s="11" t="s">
-        <v>162</v>
+      <c r="D83" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E83" s="3" t="s">
+        <v>149</v>
       </c>
       <c r="F83" s="3"/>
       <c r="G83" s="3"/>
@@ -4664,16 +4779,16 @@
         <v>147</v>
       </c>
       <c r="B84" s="10" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="C84" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D84" s="10" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
       <c r="E84" s="11" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
       <c r="F84" s="3"/>
       <c r="G84" s="3"/>
@@ -4701,20 +4816,20 @@
       <c r="AC84" s="3"/>
     </row>
     <row r="85" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A85" s="1" t="s">
+      <c r="A85" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B85" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="C85" s="1" t="s">
+      <c r="B85" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="C85" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D85" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="E85" s="11" t="s">
-        <v>166</v>
+      <c r="D85" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="E85" s="3" t="s">
+        <v>153</v>
       </c>
       <c r="F85" s="3"/>
       <c r="G85" s="3"/>
@@ -4742,20 +4857,20 @@
       <c r="AC85" s="3"/>
     </row>
     <row r="86" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A86" s="12" t="s">
+      <c r="A86" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B86" s="13" t="s">
-        <v>305</v>
-      </c>
-      <c r="C86" s="12" t="s">
+      <c r="B86" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D86" s="13" t="s">
-        <v>305</v>
-      </c>
-      <c r="E86" s="13" t="s">
-        <v>306</v>
+      <c r="D86" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E86" s="3" t="s">
+        <v>154</v>
       </c>
       <c r="F86" s="3"/>
       <c r="G86" s="3"/>
@@ -4787,16 +4902,16 @@
         <v>147</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>147</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E87" s="11" t="s">
-        <v>168</v>
+        <v>156</v>
+      </c>
+      <c r="E87" s="3" t="s">
+        <v>157</v>
       </c>
       <c r="F87" s="3"/>
       <c r="G87" s="3"/>
@@ -4824,20 +4939,20 @@
       <c r="AC87" s="3"/>
     </row>
     <row r="88" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A88" s="1" t="s">
+      <c r="A88" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B88" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="C88" s="1" t="s">
+      <c r="B88" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="C88" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D88" s="3" t="s">
-        <v>169</v>
+      <c r="D88" s="10" t="s">
+        <v>159</v>
       </c>
       <c r="E88" s="11" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="F88" s="3"/>
       <c r="G88" s="3"/>
@@ -4865,20 +4980,20 @@
       <c r="AC88" s="3"/>
     </row>
     <row r="89" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A89" s="1" t="s">
+      <c r="A89" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B89" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C89" s="1" t="s">
+      <c r="B89" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="C89" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D89" s="3" t="s">
-        <v>171</v>
+      <c r="D89" s="10" t="s">
+        <v>161</v>
       </c>
       <c r="E89" s="11" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="F89" s="3"/>
       <c r="G89" s="3"/>
@@ -4910,16 +5025,16 @@
         <v>147</v>
       </c>
       <c r="B90" s="10" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="C90" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D90" s="10" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="E90" s="11" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="F90" s="3"/>
       <c r="G90" s="3"/>
@@ -4947,20 +5062,20 @@
       <c r="AC90" s="3"/>
     </row>
     <row r="91" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A91" s="12" t="s">
+      <c r="A91" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B91" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="C91" s="12" t="s">
+      <c r="B91" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D91" s="13" t="s">
-        <v>307</v>
-      </c>
-      <c r="E91" s="13" t="s">
-        <v>308</v>
+      <c r="D91" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E91" s="11" t="s">
+        <v>166</v>
       </c>
       <c r="F91" s="3"/>
       <c r="G91" s="3"/>
@@ -4988,20 +5103,20 @@
       <c r="AC91" s="3"/>
     </row>
     <row r="92" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A92" s="9" t="s">
+      <c r="A92" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B92" s="23" t="s">
-        <v>175</v>
-      </c>
-      <c r="C92" s="9" t="s">
+      <c r="B92" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="C92" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D92" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="E92" s="24" t="s">
-        <v>177</v>
+      <c r="D92" s="13" t="s">
+        <v>305</v>
+      </c>
+      <c r="E92" s="13" t="s">
+        <v>306</v>
       </c>
       <c r="F92" s="3"/>
       <c r="G92" s="3"/>
@@ -5029,20 +5144,20 @@
       <c r="AC92" s="3"/>
     </row>
     <row r="93" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A93" s="9" t="s">
+      <c r="A93" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B93" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="C93" s="9" t="s">
+      <c r="B93" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D93" s="23" t="s">
-        <v>178</v>
-      </c>
-      <c r="E93" s="24" t="s">
-        <v>179</v>
+      <c r="D93" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E93" s="11" t="s">
+        <v>168</v>
       </c>
       <c r="F93" s="3"/>
       <c r="G93" s="3"/>
@@ -5073,17 +5188,17 @@
       <c r="A94" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B94" s="7" t="s">
-        <v>180</v>
+      <c r="B94" s="3" t="s">
+        <v>169</v>
       </c>
       <c r="C94" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D94" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="E94" s="18" t="s">
-        <v>182</v>
+      <c r="D94" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E94" s="11" t="s">
+        <v>170</v>
       </c>
       <c r="F94" s="3"/>
       <c r="G94" s="3"/>
@@ -5111,20 +5226,20 @@
       <c r="AC94" s="3"/>
     </row>
     <row r="95" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A95" s="25" t="s">
+      <c r="A95" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B95" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="C95" s="25" t="s">
+      <c r="B95" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="D95" s="26" t="s">
-        <v>184</v>
+      <c r="D95" s="3" t="s">
+        <v>171</v>
       </c>
       <c r="E95" s="11" t="s">
-        <v>185</v>
+        <v>172</v>
       </c>
       <c r="F95" s="3"/>
       <c r="G95" s="3"/>
@@ -5156,16 +5271,16 @@
         <v>147</v>
       </c>
       <c r="B96" s="10" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="C96" s="9" t="s">
         <v>147</v>
       </c>
       <c r="D96" s="10" t="s">
-        <v>187</v>
+        <v>173</v>
       </c>
       <c r="E96" s="11" t="s">
-        <v>188</v>
+        <v>174</v>
       </c>
       <c r="F96" s="3"/>
       <c r="G96" s="3"/>
@@ -5193,20 +5308,20 @@
       <c r="AC96" s="3"/>
     </row>
     <row r="97" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A97" s="1" t="s">
+      <c r="A97" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="B97" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="C97" s="1" t="s">
+      <c r="B97" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="C97" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="D97" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="E97" s="11" t="s">
-        <v>191</v>
+      <c r="D97" s="13" t="s">
+        <v>307</v>
+      </c>
+      <c r="E97" s="13" t="s">
+        <v>308</v>
       </c>
       <c r="F97" s="3"/>
       <c r="G97" s="3"/>
@@ -5234,20 +5349,20 @@
       <c r="AC97" s="3"/>
     </row>
     <row r="98" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A98" s="1" t="s">
+      <c r="A98" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="B98" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="C98" s="1" t="s">
+      <c r="B98" s="23" t="s">
+        <v>175</v>
+      </c>
+      <c r="C98" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="D98" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="E98" s="11" t="s">
-        <v>193</v>
+      <c r="D98" s="23" t="s">
+        <v>176</v>
+      </c>
+      <c r="E98" s="24" t="s">
+        <v>177</v>
       </c>
       <c r="F98" s="3"/>
       <c r="G98" s="3"/>
@@ -5275,20 +5390,20 @@
       <c r="AC98" s="3"/>
     </row>
     <row r="99" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A99" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="B99" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="D99" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="E99" s="11" t="s">
-        <v>197</v>
+      <c r="A99" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="B99" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="C99" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D99" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="E99" s="24" t="s">
+        <v>179</v>
       </c>
       <c r="F99" s="3"/>
       <c r="G99" s="3"/>
@@ -5317,15 +5432,19 @@
     </row>
     <row r="100" spans="1:29" ht="15.75" customHeight="1">
       <c r="A100" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="B100" s="3"/>
+        <v>147</v>
+      </c>
+      <c r="B100" s="7" t="s">
+        <v>180</v>
+      </c>
       <c r="C100" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="D100" s="3"/>
-      <c r="E100" s="11" t="s">
-        <v>200</v>
+        <v>147</v>
+      </c>
+      <c r="D100" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="E100" s="18" t="s">
+        <v>182</v>
       </c>
       <c r="F100" s="3"/>
       <c r="G100" s="3"/>
@@ -5354,15 +5473,19 @@
     </row>
     <row r="101" spans="1:29" ht="15.75" customHeight="1">
       <c r="A101" s="25" t="s">
-        <v>201</v>
-      </c>
-      <c r="B101" s="26"/>
+        <v>147</v>
+      </c>
+      <c r="B101" s="26" t="s">
+        <v>183</v>
+      </c>
       <c r="C101" s="25" t="s">
-        <v>201</v>
-      </c>
-      <c r="D101" s="26"/>
-      <c r="E101" s="3" t="s">
-        <v>202</v>
+        <v>147</v>
+      </c>
+      <c r="D101" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="E101" s="11" t="s">
+        <v>185</v>
       </c>
       <c r="F101" s="3"/>
       <c r="G101" s="3"/>
@@ -5391,15 +5514,19 @@
     </row>
     <row r="102" spans="1:29" ht="15.75" customHeight="1">
       <c r="A102" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="B102" s="10"/>
+        <v>147</v>
+      </c>
+      <c r="B102" s="10" t="s">
+        <v>186</v>
+      </c>
       <c r="C102" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="D102" s="10"/>
+        <v>147</v>
+      </c>
+      <c r="D102" s="10" t="s">
+        <v>187</v>
+      </c>
       <c r="E102" s="11" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="F102" s="3"/>
       <c r="G102" s="3"/>
@@ -5428,15 +5555,19 @@
     </row>
     <row r="103" spans="1:29" ht="15.75" customHeight="1">
       <c r="A103" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="B103" s="3"/>
+        <v>147</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>189</v>
+      </c>
       <c r="C103" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="D103" s="3"/>
-      <c r="E103" s="3" t="s">
-        <v>206</v>
+        <v>147</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E103" s="11" t="s">
+        <v>191</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
@@ -5465,19 +5596,19 @@
     </row>
     <row r="104" spans="1:29" ht="15.75" customHeight="1">
       <c r="A104" s="1" t="s">
-        <v>207</v>
+        <v>147</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>167</v>
+        <v>192</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>208</v>
+        <v>147</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E104" s="3" t="s">
-        <v>209</v>
+        <v>192</v>
+      </c>
+      <c r="E104" s="11" t="s">
+        <v>193</v>
       </c>
       <c r="F104" s="3"/>
       <c r="G104" s="3"/>
@@ -5506,19 +5637,19 @@
     </row>
     <row r="105" spans="1:29" ht="15.75" customHeight="1">
       <c r="A105" s="1" t="s">
-        <v>207</v>
+        <v>194</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>208</v>
+        <v>194</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="E105" s="3" t="s">
-        <v>211</v>
+        <v>196</v>
+      </c>
+      <c r="E105" s="11" t="s">
+        <v>197</v>
       </c>
       <c r="F105" s="3"/>
       <c r="G105" s="3"/>
@@ -5546,20 +5677,16 @@
       <c r="AC105" s="3"/>
     </row>
     <row r="106" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A106" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="B106" s="10" t="s">
-        <v>165</v>
-      </c>
+      <c r="A106" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="B106" s="3"/>
       <c r="C106" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="D106" s="10" t="s">
-        <v>165</v>
-      </c>
-      <c r="E106" s="10" t="s">
-        <v>212</v>
+        <v>199</v>
+      </c>
+      <c r="D106" s="3"/>
+      <c r="E106" s="11" t="s">
+        <v>200</v>
       </c>
       <c r="F106" s="3"/>
       <c r="G106" s="3"/>
@@ -5587,20 +5714,16 @@
       <c r="AC106" s="3"/>
     </row>
     <row r="107" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A107" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="B107" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="C107" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="D107" s="3" t="s">
-        <v>214</v>
-      </c>
+      <c r="A107" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="B107" s="26"/>
+      <c r="C107" s="25" t="s">
+        <v>201</v>
+      </c>
+      <c r="D107" s="26"/>
       <c r="E107" s="3" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="F107" s="3"/>
       <c r="G107" s="3"/>
@@ -5628,20 +5751,16 @@
       <c r="AC107" s="3"/>
     </row>
     <row r="108" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A108" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="B108" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="D108" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E108" s="3" t="s">
-        <v>216</v>
+      <c r="A108" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="B108" s="10"/>
+      <c r="C108" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="D108" s="10"/>
+      <c r="E108" s="11" t="s">
+        <v>204</v>
       </c>
       <c r="F108" s="3"/>
       <c r="G108" s="3"/>
@@ -5669,20 +5788,16 @@
       <c r="AC108" s="3"/>
     </row>
     <row r="109" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A109" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="B109" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="C109" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="D109" s="3" t="s">
-        <v>217</v>
-      </c>
+      <c r="A109" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B109" s="3"/>
+      <c r="C109" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D109" s="3"/>
       <c r="E109" s="3" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
       <c r="F109" s="3"/>
       <c r="G109" s="3"/>
@@ -5711,19 +5826,19 @@
     </row>
     <row r="110" spans="1:29" ht="15.75" customHeight="1">
       <c r="A110" s="1" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>219</v>
+        <v>167</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>219</v>
+        <v>167</v>
       </c>
       <c r="E110" s="3" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="F110" s="3"/>
       <c r="G110" s="3"/>
@@ -5751,16 +5866,20 @@
       <c r="AC110" s="3"/>
     </row>
     <row r="111" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A111" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="B111" s="10"/>
-      <c r="C111" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="D111" s="10"/>
-      <c r="E111" s="11" t="s">
-        <v>222</v>
+      <c r="A111" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B111" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="E111" s="3" t="s">
+        <v>211</v>
       </c>
       <c r="F111" s="3"/>
       <c r="G111" s="3"/>
@@ -5788,16 +5907,20 @@
       <c r="AC111" s="3"/>
     </row>
     <row r="112" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A112" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="B112" s="13"/>
-      <c r="C112" s="12" t="s">
-        <v>309</v>
-      </c>
-      <c r="D112" s="13"/>
-      <c r="E112" s="13" t="s">
-        <v>310</v>
+      <c r="A112" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B112" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="D112" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="E112" s="10" t="s">
+        <v>212</v>
       </c>
       <c r="F112" s="3"/>
       <c r="G112" s="3"/>
@@ -5826,15 +5949,19 @@
     </row>
     <row r="113" spans="1:29" ht="15.75" customHeight="1">
       <c r="A113" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="B113" s="3"/>
+        <v>213</v>
+      </c>
+      <c r="B113" s="3" t="s">
+        <v>214</v>
+      </c>
       <c r="C113" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="D113" s="3"/>
+        <v>213</v>
+      </c>
+      <c r="D113" s="3" t="s">
+        <v>214</v>
+      </c>
       <c r="E113" s="3" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="F113" s="3"/>
       <c r="G113" s="3"/>
@@ -5863,19 +5990,19 @@
     </row>
     <row r="114" spans="1:29" ht="15.75" customHeight="1">
       <c r="A114" s="3" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>225</v>
+        <v>57</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>226</v>
+        <v>57</v>
       </c>
       <c r="E114" s="3" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="F114" s="3"/>
       <c r="G114" s="3"/>
@@ -5903,20 +6030,20 @@
       <c r="AC114" s="3"/>
     </row>
     <row r="115" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A115" s="1" t="s">
-        <v>223</v>
+      <c r="A115" s="3" t="s">
+        <v>213</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>223</v>
+        <v>217</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>213</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="E115" s="3" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="F115" s="3"/>
       <c r="G115" s="3"/>
@@ -5944,16 +6071,20 @@
       <c r="AC115" s="3"/>
     </row>
     <row r="116" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A116" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="B116" s="10"/>
-      <c r="C116" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="D116" s="10"/>
+      <c r="A116" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="D116" s="3" t="s">
+        <v>219</v>
+      </c>
       <c r="E116" s="3" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="F116" s="3"/>
       <c r="G116" s="3"/>
@@ -5981,16 +6112,16 @@
       <c r="AC116" s="3"/>
     </row>
     <row r="117" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A117" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B117" s="3"/>
-      <c r="C117" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D117" s="3"/>
-      <c r="E117" s="3" t="s">
-        <v>232</v>
+      <c r="A117" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="B117" s="10"/>
+      <c r="C117" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="D117" s="10"/>
+      <c r="E117" s="11" t="s">
+        <v>222</v>
       </c>
       <c r="F117" s="3"/>
       <c r="G117" s="3"/>
@@ -6018,20 +6149,20 @@
       <c r="AC117" s="3"/>
     </row>
     <row r="118" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A118" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B118" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="E118" s="3" t="s">
-        <v>235</v>
+      <c r="A118" s="30" t="s">
+        <v>320</v>
+      </c>
+      <c r="B118" s="31" t="s">
+        <v>321</v>
+      </c>
+      <c r="C118" s="30" t="s">
+        <v>322</v>
+      </c>
+      <c r="D118" s="31" t="s">
+        <v>321</v>
+      </c>
+      <c r="E118" s="32" t="s">
+        <v>323</v>
       </c>
       <c r="F118" s="3"/>
       <c r="G118" s="3"/>
@@ -6059,20 +6190,20 @@
       <c r="AC118" s="3"/>
     </row>
     <row r="119" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A119" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B119" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="E119" s="3" t="s">
-        <v>237</v>
+      <c r="A119" s="30" t="s">
+        <v>320</v>
+      </c>
+      <c r="B119" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="C119" s="30" t="s">
+        <v>322</v>
+      </c>
+      <c r="D119" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="E119" s="32" t="s">
+        <v>325</v>
       </c>
       <c r="F119" s="3"/>
       <c r="G119" s="3"/>
@@ -6100,20 +6231,16 @@
       <c r="AC119" s="3"/>
     </row>
     <row r="120" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A120" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B120" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D120" s="3" t="s">
-        <v>239</v>
-      </c>
-      <c r="E120" s="3" t="s">
-        <v>240</v>
+      <c r="A120" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="B120" s="13"/>
+      <c r="C120" s="12" t="s">
+        <v>309</v>
+      </c>
+      <c r="D120" s="13"/>
+      <c r="E120" s="13" t="s">
+        <v>310</v>
       </c>
       <c r="F120" s="3"/>
       <c r="G120" s="3"/>
@@ -6142,19 +6269,15 @@
     </row>
     <row r="121" spans="1:29" ht="15.75" customHeight="1">
       <c r="A121" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B121" s="3" t="s">
-        <v>241</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="B121" s="3"/>
       <c r="C121" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D121" s="3" t="s">
-        <v>242</v>
-      </c>
+        <v>223</v>
+      </c>
+      <c r="D121" s="3"/>
       <c r="E121" s="3" t="s">
-        <v>243</v>
+        <v>224</v>
       </c>
       <c r="F121" s="3"/>
       <c r="G121" s="3"/>
@@ -6182,20 +6305,20 @@
       <c r="AC121" s="3"/>
     </row>
     <row r="122" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A122" s="1" t="s">
-        <v>210</v>
+      <c r="A122" s="3" t="s">
+        <v>223</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="C122" s="1" t="s">
-        <v>210</v>
+        <v>225</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>223</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>245</v>
+        <v>226</v>
       </c>
       <c r="E122" s="3" t="s">
-        <v>246</v>
+        <v>227</v>
       </c>
       <c r="F122" s="3"/>
       <c r="G122" s="3"/>
@@ -6224,19 +6347,19 @@
     </row>
     <row r="123" spans="1:29" ht="15.75" customHeight="1">
       <c r="A123" s="1" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>247</v>
+        <v>228</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>210</v>
+        <v>223</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>248</v>
+        <v>228</v>
       </c>
       <c r="E123" s="3" t="s">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="F123" s="3"/>
       <c r="G123" s="3"/>
@@ -6264,20 +6387,16 @@
       <c r="AC123" s="3"/>
     </row>
     <row r="124" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A124" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="B124" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="C124" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>250</v>
-      </c>
+      <c r="A124" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="B124" s="10"/>
+      <c r="C124" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="D124" s="10"/>
       <c r="E124" s="3" t="s">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="F124" s="3"/>
       <c r="G124" s="3"/>
@@ -6308,17 +6427,13 @@
       <c r="A125" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B125" s="3" t="s">
-        <v>252</v>
-      </c>
+      <c r="B125" s="3"/>
       <c r="C125" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="D125" s="3" t="s">
-        <v>252</v>
-      </c>
+      <c r="D125" s="3"/>
       <c r="E125" s="3" t="s">
-        <v>253</v>
+        <v>232</v>
       </c>
       <c r="F125" s="3"/>
       <c r="G125" s="3"/>
@@ -6350,16 +6465,16 @@
         <v>210</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>254</v>
+        <v>233</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>255</v>
+        <v>234</v>
       </c>
       <c r="E126" s="3" t="s">
-        <v>256</v>
+        <v>235</v>
       </c>
       <c r="F126" s="3"/>
       <c r="G126" s="3"/>
@@ -6391,16 +6506,16 @@
         <v>210</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>257</v>
+        <v>236</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>257</v>
+        <v>236</v>
       </c>
       <c r="E127" s="3" t="s">
-        <v>258</v>
+        <v>237</v>
       </c>
       <c r="F127" s="3"/>
       <c r="G127" s="3"/>
@@ -6432,16 +6547,16 @@
         <v>210</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>259</v>
+        <v>238</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="E128" s="3" t="s">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="F128" s="3"/>
       <c r="G128" s="3"/>
@@ -6473,16 +6588,16 @@
         <v>210</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>261</v>
+        <v>241</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>210</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>261</v>
+        <v>242</v>
       </c>
       <c r="E129" s="3" t="s">
-        <v>262</v>
+        <v>243</v>
       </c>
       <c r="F129" s="3"/>
       <c r="G129" s="3"/>
@@ -6510,16 +6625,20 @@
       <c r="AC129" s="3"/>
     </row>
     <row r="130" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A130" s="25" t="s">
-        <v>311</v>
-      </c>
-      <c r="B130" s="26"/>
-      <c r="C130" s="25" t="s">
-        <v>311</v>
-      </c>
-      <c r="D130" s="26"/>
+      <c r="A130" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>245</v>
+      </c>
       <c r="E130" s="3" t="s">
-        <v>312</v>
+        <v>246</v>
       </c>
       <c r="F130" s="3"/>
       <c r="G130" s="3"/>
@@ -6547,16 +6666,20 @@
       <c r="AC130" s="3"/>
     </row>
     <row r="131" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A131" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="B131" s="10"/>
-      <c r="C131" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="D131" s="10"/>
+      <c r="A131" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>248</v>
+      </c>
       <c r="E131" s="3" t="s">
-        <v>264</v>
+        <v>249</v>
       </c>
       <c r="F131" s="3"/>
       <c r="G131" s="3"/>
@@ -6585,15 +6708,19 @@
     </row>
     <row r="132" spans="1:29" ht="15.75" customHeight="1">
       <c r="A132" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="B132" s="3"/>
+        <v>210</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>250</v>
+      </c>
       <c r="C132" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="D132" s="3"/>
+        <v>210</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>250</v>
+      </c>
       <c r="E132" s="3" t="s">
-        <v>266</v>
+        <v>251</v>
       </c>
       <c r="F132" s="3"/>
       <c r="G132" s="3"/>
@@ -6622,15 +6749,19 @@
     </row>
     <row r="133" spans="1:29" ht="15.75" customHeight="1">
       <c r="A133" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="B133" s="3"/>
+        <v>210</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="C133" s="1" t="s">
-        <v>267</v>
-      </c>
-      <c r="D133" s="3"/>
+        <v>210</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>252</v>
+      </c>
       <c r="E133" s="3" t="s">
-        <v>268</v>
+        <v>253</v>
       </c>
       <c r="F133" s="3"/>
       <c r="G133" s="3"/>
@@ -6658,11 +6789,21 @@
       <c r="AC133" s="3"/>
     </row>
     <row r="134" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A134" s="3"/>
-      <c r="B134" s="3"/>
-      <c r="C134" s="3"/>
-      <c r="D134" s="3"/>
-      <c r="E134" s="3"/>
+      <c r="A134" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D134" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="E134" s="3" t="s">
+        <v>256</v>
+      </c>
       <c r="F134" s="3"/>
       <c r="G134" s="3"/>
       <c r="H134" s="3"/>
@@ -6689,11 +6830,21 @@
       <c r="AC134" s="3"/>
     </row>
     <row r="135" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A135" s="1"/>
-      <c r="B135" s="3"/>
-      <c r="C135" s="3"/>
-      <c r="D135" s="3"/>
-      <c r="E135" s="3"/>
+      <c r="A135" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D135" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E135" s="3" t="s">
+        <v>258</v>
+      </c>
       <c r="F135" s="3"/>
       <c r="G135" s="3"/>
       <c r="H135" s="3"/>
@@ -6720,11 +6871,21 @@
       <c r="AC135" s="3"/>
     </row>
     <row r="136" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A136" s="3"/>
-      <c r="B136" s="3"/>
-      <c r="C136" s="3"/>
-      <c r="D136" s="3"/>
-      <c r="E136" s="3"/>
+      <c r="A136" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="E136" s="3" t="s">
+        <v>260</v>
+      </c>
       <c r="F136" s="3"/>
       <c r="G136" s="3"/>
       <c r="H136" s="3"/>
@@ -6751,11 +6912,21 @@
       <c r="AC136" s="3"/>
     </row>
     <row r="137" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A137" s="1"/>
-      <c r="B137" s="3"/>
-      <c r="C137" s="3"/>
-      <c r="D137" s="3"/>
-      <c r="E137" s="3"/>
+      <c r="A137" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="D137" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="E137" s="3" t="s">
+        <v>262</v>
+      </c>
       <c r="F137" s="3"/>
       <c r="G137" s="3"/>
       <c r="H137" s="3"/>
@@ -6782,11 +6953,17 @@
       <c r="AC137" s="3"/>
     </row>
     <row r="138" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A138" s="3"/>
-      <c r="B138" s="3"/>
-      <c r="C138" s="3"/>
-      <c r="D138" s="3"/>
-      <c r="E138" s="3"/>
+      <c r="A138" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="B138" s="26"/>
+      <c r="C138" s="25" t="s">
+        <v>311</v>
+      </c>
+      <c r="D138" s="26"/>
+      <c r="E138" s="3" t="s">
+        <v>312</v>
+      </c>
       <c r="F138" s="3"/>
       <c r="G138" s="3"/>
       <c r="H138" s="3"/>
@@ -6813,11 +6990,17 @@
       <c r="AC138" s="3"/>
     </row>
     <row r="139" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A139" s="3"/>
-      <c r="B139" s="3"/>
-      <c r="C139" s="3"/>
-      <c r="D139" s="3"/>
-      <c r="E139" s="3"/>
+      <c r="A139" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="B139" s="10"/>
+      <c r="C139" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="D139" s="10"/>
+      <c r="E139" s="3" t="s">
+        <v>264</v>
+      </c>
       <c r="F139" s="3"/>
       <c r="G139" s="3"/>
       <c r="H139" s="3"/>
@@ -6844,11 +7027,17 @@
       <c r="AC139" s="3"/>
     </row>
     <row r="140" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A140" s="3"/>
+      <c r="A140" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="B140" s="3"/>
-      <c r="C140" s="3"/>
+      <c r="C140" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="D140" s="3"/>
-      <c r="E140" s="3"/>
+      <c r="E140" s="3" t="s">
+        <v>266</v>
+      </c>
       <c r="F140" s="3"/>
       <c r="G140" s="3"/>
       <c r="H140" s="3"/>
@@ -6875,11 +7064,17 @@
       <c r="AC140" s="3"/>
     </row>
     <row r="141" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A141" s="3"/>
+      <c r="A141" s="1" t="s">
+        <v>267</v>
+      </c>
       <c r="B141" s="3"/>
-      <c r="C141" s="3"/>
+      <c r="C141" s="1" t="s">
+        <v>267</v>
+      </c>
       <c r="D141" s="3"/>
-      <c r="E141" s="3"/>
+      <c r="E141" s="3" t="s">
+        <v>268</v>
+      </c>
       <c r="F141" s="3"/>
       <c r="G141" s="3"/>
       <c r="H141" s="3"/>
@@ -6905,67 +7100,79 @@
       <c r="AB141" s="3"/>
       <c r="AC141" s="3"/>
     </row>
-    <row r="142" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A142" s="3"/>
-      <c r="B142" s="3"/>
-      <c r="C142" s="3"/>
-      <c r="D142" s="3"/>
-      <c r="E142" s="3"/>
-      <c r="F142" s="3"/>
-      <c r="G142" s="3"/>
-      <c r="H142" s="3"/>
-      <c r="I142" s="3"/>
-      <c r="J142" s="3"/>
-      <c r="K142" s="3"/>
-      <c r="L142" s="3"/>
-      <c r="M142" s="3"/>
-      <c r="N142" s="3"/>
-      <c r="O142" s="3"/>
-      <c r="P142" s="3"/>
-      <c r="Q142" s="3"/>
-      <c r="R142" s="3"/>
-      <c r="S142" s="3"/>
-      <c r="T142" s="3"/>
-      <c r="U142" s="3"/>
-      <c r="V142" s="3"/>
-      <c r="W142" s="3"/>
-      <c r="X142" s="3"/>
-      <c r="Y142" s="3"/>
-      <c r="Z142" s="3"/>
-      <c r="AA142" s="3"/>
-      <c r="AB142" s="3"/>
-      <c r="AC142" s="3"/>
-    </row>
-    <row r="143" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A143" s="3"/>
-      <c r="B143" s="3"/>
-      <c r="C143" s="3"/>
-      <c r="D143" s="3"/>
-      <c r="E143" s="3"/>
-      <c r="F143" s="3"/>
-      <c r="G143" s="3"/>
-      <c r="H143" s="3"/>
-      <c r="I143" s="3"/>
-      <c r="J143" s="3"/>
-      <c r="K143" s="3"/>
-      <c r="L143" s="3"/>
-      <c r="M143" s="3"/>
-      <c r="N143" s="3"/>
-      <c r="O143" s="3"/>
-      <c r="P143" s="3"/>
-      <c r="Q143" s="3"/>
-      <c r="R143" s="3"/>
-      <c r="S143" s="3"/>
-      <c r="T143" s="3"/>
-      <c r="U143" s="3"/>
-      <c r="V143" s="3"/>
-      <c r="W143" s="3"/>
-      <c r="X143" s="3"/>
-      <c r="Y143" s="3"/>
-      <c r="Z143" s="3"/>
-      <c r="AA143" s="3"/>
-      <c r="AB143" s="3"/>
-      <c r="AC143" s="3"/>
+    <row r="142" spans="1:29" s="29" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A142" s="28" t="s">
+        <v>315</v>
+      </c>
+      <c r="B142" s="28"/>
+      <c r="C142" s="28" t="s">
+        <v>316</v>
+      </c>
+      <c r="D142" s="28"/>
+      <c r="E142" s="28" t="s">
+        <v>317</v>
+      </c>
+      <c r="F142" s="28"/>
+      <c r="G142" s="28"/>
+      <c r="H142" s="28"/>
+      <c r="I142" s="28"/>
+      <c r="J142" s="28"/>
+      <c r="K142" s="28"/>
+      <c r="L142" s="28"/>
+      <c r="M142" s="28"/>
+      <c r="N142" s="28"/>
+      <c r="O142" s="28"/>
+      <c r="P142" s="28"/>
+      <c r="Q142" s="28"/>
+      <c r="R142" s="28"/>
+      <c r="S142" s="28"/>
+      <c r="T142" s="28"/>
+      <c r="U142" s="28"/>
+      <c r="V142" s="28"/>
+      <c r="W142" s="28"/>
+      <c r="X142" s="28"/>
+      <c r="Y142" s="28"/>
+      <c r="Z142" s="28"/>
+      <c r="AA142" s="28"/>
+      <c r="AB142" s="28"/>
+      <c r="AC142" s="28"/>
+    </row>
+    <row r="143" spans="1:29" s="29" customFormat="1" ht="15.75" customHeight="1">
+      <c r="A143" s="27" t="s">
+        <v>318</v>
+      </c>
+      <c r="B143" s="28"/>
+      <c r="C143" s="28" t="s">
+        <v>318</v>
+      </c>
+      <c r="D143" s="28"/>
+      <c r="E143" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="F143" s="28"/>
+      <c r="G143" s="28"/>
+      <c r="H143" s="28"/>
+      <c r="I143" s="28"/>
+      <c r="J143" s="28"/>
+      <c r="K143" s="28"/>
+      <c r="L143" s="28"/>
+      <c r="M143" s="28"/>
+      <c r="N143" s="28"/>
+      <c r="O143" s="28"/>
+      <c r="P143" s="28"/>
+      <c r="Q143" s="28"/>
+      <c r="R143" s="28"/>
+      <c r="S143" s="28"/>
+      <c r="T143" s="28"/>
+      <c r="U143" s="28"/>
+      <c r="V143" s="28"/>
+      <c r="W143" s="28"/>
+      <c r="X143" s="28"/>
+      <c r="Y143" s="28"/>
+      <c r="Z143" s="28"/>
+      <c r="AA143" s="28"/>
+      <c r="AB143" s="28"/>
+      <c r="AC143" s="28"/>
     </row>
     <row r="144" spans="1:29" ht="15.75" customHeight="1">
       <c r="A144" s="3"/>
@@ -6999,7 +7206,7 @@
       <c r="AC144" s="3"/>
     </row>
     <row r="145" spans="1:29" ht="15.75" customHeight="1">
-      <c r="A145" s="3"/>
+      <c r="A145" s="1"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
       <c r="D145" s="3"/>
@@ -35177,6 +35384,254 @@
       <c r="AB1053" s="3"/>
       <c r="AC1053" s="3"/>
     </row>
+    <row r="1054" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1054" s="3"/>
+      <c r="B1054" s="3"/>
+      <c r="C1054" s="3"/>
+      <c r="D1054" s="3"/>
+      <c r="E1054" s="3"/>
+      <c r="F1054" s="3"/>
+      <c r="G1054" s="3"/>
+      <c r="H1054" s="3"/>
+      <c r="I1054" s="3"/>
+      <c r="J1054" s="3"/>
+      <c r="K1054" s="3"/>
+      <c r="L1054" s="3"/>
+      <c r="M1054" s="3"/>
+      <c r="N1054" s="3"/>
+      <c r="O1054" s="3"/>
+      <c r="P1054" s="3"/>
+      <c r="Q1054" s="3"/>
+      <c r="R1054" s="3"/>
+      <c r="S1054" s="3"/>
+      <c r="T1054" s="3"/>
+      <c r="U1054" s="3"/>
+      <c r="V1054" s="3"/>
+      <c r="W1054" s="3"/>
+      <c r="X1054" s="3"/>
+      <c r="Y1054" s="3"/>
+      <c r="Z1054" s="3"/>
+      <c r="AA1054" s="3"/>
+      <c r="AB1054" s="3"/>
+      <c r="AC1054" s="3"/>
+    </row>
+    <row r="1055" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1055" s="3"/>
+      <c r="B1055" s="3"/>
+      <c r="C1055" s="3"/>
+      <c r="D1055" s="3"/>
+      <c r="E1055" s="3"/>
+      <c r="F1055" s="3"/>
+      <c r="G1055" s="3"/>
+      <c r="H1055" s="3"/>
+      <c r="I1055" s="3"/>
+      <c r="J1055" s="3"/>
+      <c r="K1055" s="3"/>
+      <c r="L1055" s="3"/>
+      <c r="M1055" s="3"/>
+      <c r="N1055" s="3"/>
+      <c r="O1055" s="3"/>
+      <c r="P1055" s="3"/>
+      <c r="Q1055" s="3"/>
+      <c r="R1055" s="3"/>
+      <c r="S1055" s="3"/>
+      <c r="T1055" s="3"/>
+      <c r="U1055" s="3"/>
+      <c r="V1055" s="3"/>
+      <c r="W1055" s="3"/>
+      <c r="X1055" s="3"/>
+      <c r="Y1055" s="3"/>
+      <c r="Z1055" s="3"/>
+      <c r="AA1055" s="3"/>
+      <c r="AB1055" s="3"/>
+      <c r="AC1055" s="3"/>
+    </row>
+    <row r="1056" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1056" s="3"/>
+      <c r="B1056" s="3"/>
+      <c r="C1056" s="3"/>
+      <c r="D1056" s="3"/>
+      <c r="E1056" s="3"/>
+      <c r="F1056" s="3"/>
+      <c r="G1056" s="3"/>
+      <c r="H1056" s="3"/>
+      <c r="I1056" s="3"/>
+      <c r="J1056" s="3"/>
+      <c r="K1056" s="3"/>
+      <c r="L1056" s="3"/>
+      <c r="M1056" s="3"/>
+      <c r="N1056" s="3"/>
+      <c r="O1056" s="3"/>
+      <c r="P1056" s="3"/>
+      <c r="Q1056" s="3"/>
+      <c r="R1056" s="3"/>
+      <c r="S1056" s="3"/>
+      <c r="T1056" s="3"/>
+      <c r="U1056" s="3"/>
+      <c r="V1056" s="3"/>
+      <c r="W1056" s="3"/>
+      <c r="X1056" s="3"/>
+      <c r="Y1056" s="3"/>
+      <c r="Z1056" s="3"/>
+      <c r="AA1056" s="3"/>
+      <c r="AB1056" s="3"/>
+      <c r="AC1056" s="3"/>
+    </row>
+    <row r="1057" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1057" s="3"/>
+      <c r="B1057" s="3"/>
+      <c r="C1057" s="3"/>
+      <c r="D1057" s="3"/>
+      <c r="E1057" s="3"/>
+      <c r="F1057" s="3"/>
+      <c r="G1057" s="3"/>
+      <c r="H1057" s="3"/>
+      <c r="I1057" s="3"/>
+      <c r="J1057" s="3"/>
+      <c r="K1057" s="3"/>
+      <c r="L1057" s="3"/>
+      <c r="M1057" s="3"/>
+      <c r="N1057" s="3"/>
+      <c r="O1057" s="3"/>
+      <c r="P1057" s="3"/>
+      <c r="Q1057" s="3"/>
+      <c r="R1057" s="3"/>
+      <c r="S1057" s="3"/>
+      <c r="T1057" s="3"/>
+      <c r="U1057" s="3"/>
+      <c r="V1057" s="3"/>
+      <c r="W1057" s="3"/>
+      <c r="X1057" s="3"/>
+      <c r="Y1057" s="3"/>
+      <c r="Z1057" s="3"/>
+      <c r="AA1057" s="3"/>
+      <c r="AB1057" s="3"/>
+      <c r="AC1057" s="3"/>
+    </row>
+    <row r="1058" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1058" s="3"/>
+      <c r="B1058" s="3"/>
+      <c r="C1058" s="3"/>
+      <c r="D1058" s="3"/>
+      <c r="E1058" s="3"/>
+      <c r="F1058" s="3"/>
+      <c r="G1058" s="3"/>
+      <c r="H1058" s="3"/>
+      <c r="I1058" s="3"/>
+      <c r="J1058" s="3"/>
+      <c r="K1058" s="3"/>
+      <c r="L1058" s="3"/>
+      <c r="M1058" s="3"/>
+      <c r="N1058" s="3"/>
+      <c r="O1058" s="3"/>
+      <c r="P1058" s="3"/>
+      <c r="Q1058" s="3"/>
+      <c r="R1058" s="3"/>
+      <c r="S1058" s="3"/>
+      <c r="T1058" s="3"/>
+      <c r="U1058" s="3"/>
+      <c r="V1058" s="3"/>
+      <c r="W1058" s="3"/>
+      <c r="X1058" s="3"/>
+      <c r="Y1058" s="3"/>
+      <c r="Z1058" s="3"/>
+      <c r="AA1058" s="3"/>
+      <c r="AB1058" s="3"/>
+      <c r="AC1058" s="3"/>
+    </row>
+    <row r="1059" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1059" s="3"/>
+      <c r="B1059" s="3"/>
+      <c r="C1059" s="3"/>
+      <c r="D1059" s="3"/>
+      <c r="E1059" s="3"/>
+      <c r="F1059" s="3"/>
+      <c r="G1059" s="3"/>
+      <c r="H1059" s="3"/>
+      <c r="I1059" s="3"/>
+      <c r="J1059" s="3"/>
+      <c r="K1059" s="3"/>
+      <c r="L1059" s="3"/>
+      <c r="M1059" s="3"/>
+      <c r="N1059" s="3"/>
+      <c r="O1059" s="3"/>
+      <c r="P1059" s="3"/>
+      <c r="Q1059" s="3"/>
+      <c r="R1059" s="3"/>
+      <c r="S1059" s="3"/>
+      <c r="T1059" s="3"/>
+      <c r="U1059" s="3"/>
+      <c r="V1059" s="3"/>
+      <c r="W1059" s="3"/>
+      <c r="X1059" s="3"/>
+      <c r="Y1059" s="3"/>
+      <c r="Z1059" s="3"/>
+      <c r="AA1059" s="3"/>
+      <c r="AB1059" s="3"/>
+      <c r="AC1059" s="3"/>
+    </row>
+    <row r="1060" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1060" s="3"/>
+      <c r="B1060" s="3"/>
+      <c r="C1060" s="3"/>
+      <c r="D1060" s="3"/>
+      <c r="E1060" s="3"/>
+      <c r="F1060" s="3"/>
+      <c r="G1060" s="3"/>
+      <c r="H1060" s="3"/>
+      <c r="I1060" s="3"/>
+      <c r="J1060" s="3"/>
+      <c r="K1060" s="3"/>
+      <c r="L1060" s="3"/>
+      <c r="M1060" s="3"/>
+      <c r="N1060" s="3"/>
+      <c r="O1060" s="3"/>
+      <c r="P1060" s="3"/>
+      <c r="Q1060" s="3"/>
+      <c r="R1060" s="3"/>
+      <c r="S1060" s="3"/>
+      <c r="T1060" s="3"/>
+      <c r="U1060" s="3"/>
+      <c r="V1060" s="3"/>
+      <c r="W1060" s="3"/>
+      <c r="X1060" s="3"/>
+      <c r="Y1060" s="3"/>
+      <c r="Z1060" s="3"/>
+      <c r="AA1060" s="3"/>
+      <c r="AB1060" s="3"/>
+      <c r="AC1060" s="3"/>
+    </row>
+    <row r="1061" spans="1:29" ht="15.75" customHeight="1">
+      <c r="A1061" s="3"/>
+      <c r="B1061" s="3"/>
+      <c r="C1061" s="3"/>
+      <c r="D1061" s="3"/>
+      <c r="E1061" s="3"/>
+      <c r="F1061" s="3"/>
+      <c r="G1061" s="3"/>
+      <c r="H1061" s="3"/>
+      <c r="I1061" s="3"/>
+      <c r="J1061" s="3"/>
+      <c r="K1061" s="3"/>
+      <c r="L1061" s="3"/>
+      <c r="M1061" s="3"/>
+      <c r="N1061" s="3"/>
+      <c r="O1061" s="3"/>
+      <c r="P1061" s="3"/>
+      <c r="Q1061" s="3"/>
+      <c r="R1061" s="3"/>
+      <c r="S1061" s="3"/>
+      <c r="T1061" s="3"/>
+      <c r="U1061" s="3"/>
+      <c r="V1061" s="3"/>
+      <c r="W1061" s="3"/>
+      <c r="X1061" s="3"/>
+      <c r="Y1061" s="3"/>
+      <c r="Z1061" s="3"/>
+      <c r="AA1061" s="3"/>
+      <c r="AB1061" s="3"/>
+      <c r="AC1061" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>

</xml_diff>